<commit_message>
For higher dimension functions the grid size becomes too large so I have tried using Latin Hypercude Sampling and Sobol in addition to Cartesian (the simple grid size) this week to find candidate points/queries. I have done this introducing a config parameter called 'sample_strategy'     sample_strategy: "lhs"   # cartesian / latin hypercube sampling (lhs) / sobol I have renamed the file containing my submissions and their outputs more sensibly.
</commit_message>
<xml_diff>
--- a/BBO_function_descriptions.xlsx
+++ b/BBO_function_descriptions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ajay.amrite/Documents/AI Course/Capstone/Black-Box functions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3A76AD0-8251-DA4C-B19D-88D6718F063B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310F906C-6829-024F-AD37-11CDD9773C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{BFE7CD30-5B71-574E-BA93-034A77AB7E86}"/>
   </bookViews>

</xml_diff>